<commit_message>
Rencontre : alignement du mapping des participants sur FRCDARencontre
La tranche autresParticipants n'existe plus dans le profil CDA : le mapping de participant
cible Encounter.participant avec le display FRCDAParticipantCorps. f53c9c41ef61e67bcfcfd01998c4c547b8d66d8f
</commit_message>
<xml_diff>
--- a/majMapping/ig/FREncounterLMCDAFHIR.xlsx
+++ b/majMapping/ig/FREncounterLMCDAFHIR.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="94">
   <si>
     <t>Property</t>
   </si>
@@ -61,7 +61,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-10-07T13:52:25+00:00</t>
+    <t>2026-10-08T12:48:01+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -166,7 +166,10 @@
     <t>FRLMEncounter.participant</t>
   </si>
   <si>
-    <t>Encounter.participant:autresParticipants</t>
+    <t>Encounter.participant</t>
+  </si>
+  <si>
+    <t>FRCDAParticipantCorps</t>
   </si>
   <si>
     <t>FRLMEncounter.serviceProvider</t>
@@ -224,9 +227,6 @@
   </si>
   <si>
     <t>Encounter.priority</t>
-  </si>
-  <si>
-    <t>Encounter.participant</t>
   </si>
   <si>
     <t>Encounter.serviceProvider</t>
@@ -692,70 +692,72 @@
       <c r="D10" t="s" s="2">
         <v>50</v>
       </c>
-      <c r="E10" s="2"/>
+      <c r="E10" t="s" s="2">
+        <v>51</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="2">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" t="s" s="2">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D11" t="s" s="2">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E11" s="2"/>
     </row>
     <row r="12">
       <c r="A12" t="s" s="2">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B12" s="2"/>
       <c r="C12" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D12" t="s" s="2">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E12" s="2"/>
     </row>
     <row r="13">
       <c r="A13" t="s" s="2">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" t="s" s="2">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D13" t="s" s="2">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E13" s="2"/>
     </row>
     <row r="14">
       <c r="A14" t="s" s="2">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" t="s" s="2">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D14" t="s" s="2">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E14" s="2"/>
     </row>
     <row r="15">
       <c r="A15" t="s" s="2">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B15" s="2"/>
       <c r="C15" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D15" t="s" s="2">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E15" s="2"/>
     </row>
@@ -797,7 +799,7 @@
         <v>31</v>
       </c>
       <c r="D2" t="s" s="2">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E2" t="s" s="2">
         <v>31</v>
@@ -815,7 +817,7 @@
         <v>35</v>
       </c>
       <c r="E3" t="s" s="2">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="4">
@@ -827,7 +829,7 @@
         <v>34</v>
       </c>
       <c r="D4" t="s" s="2">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E4" s="2"/>
     </row>
@@ -840,7 +842,7 @@
         <v>34</v>
       </c>
       <c r="D5" t="s" s="2">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E5" s="2"/>
     </row>
@@ -853,7 +855,7 @@
         <v>34</v>
       </c>
       <c r="D6" t="s" s="2">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E6" s="2"/>
     </row>
@@ -866,7 +868,7 @@
         <v>34</v>
       </c>
       <c r="D7" t="s" s="2">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E7" s="2"/>
     </row>
@@ -879,7 +881,7 @@
         <v>34</v>
       </c>
       <c r="D8" t="s" s="2">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E8" s="2"/>
     </row>
@@ -892,7 +894,7 @@
         <v>34</v>
       </c>
       <c r="D9" t="s" s="2">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E9" s="2"/>
     </row>
@@ -905,13 +907,13 @@
         <v>34</v>
       </c>
       <c r="D10" t="s" s="2">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="E10" s="2"/>
     </row>
     <row r="11">
       <c r="A11" t="s" s="2">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" t="s" s="2">
@@ -924,7 +926,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s" s="2">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B12" s="2"/>
       <c r="C12" t="s" s="2">
@@ -954,7 +956,7 @@
       </c>
       <c r="B14" s="2"/>
       <c r="C14" t="s" s="2">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D14" t="s" s="2">
         <v>76</v>
@@ -967,7 +969,7 @@
       </c>
       <c r="B15" s="2"/>
       <c r="C15" t="s" s="2">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D15" t="s" s="2">
         <v>78</v>
@@ -1006,7 +1008,7 @@
       </c>
       <c r="B18" s="2"/>
       <c r="C18" t="s" s="2">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D18" t="s" s="2">
         <v>83</v>
@@ -1041,7 +1043,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s" s="2">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B21" s="2"/>
       <c r="C21" t="s" s="2">
@@ -1067,7 +1069,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s" s="2">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B23" s="2"/>
       <c r="C23" t="s" s="2">

</xml_diff>